<commit_message>
Correction nom bundle 5f49eb20f7b0c2722fce5ec349e32c2b66f6f3bd
</commit_message>
<xml_diff>
--- a/ig/travaux-tru/all-profiles.xlsx
+++ b/ig/travaux-tru/all-profiles.xlsx
@@ -3449,24 +3449,22 @@
     <t>Task outputs can take any form.</t>
   </si>
   <si>
-    <t>esms-bundle-resultat-recherche-notification-esms</t>
-  </si>
-  <si>
-    <t>https://interop.esante.gouv.fr/ig/fhir/sdo/StructureDefinition/esms-bundle-resultat-recherche-notification-esms</t>
-  </si>
-  <si>
-    <t>ESMSBundleResultatRechercheNotificationESMS</t>
+    <t>sdo-bundle-resultat-recherche-notification-esms</t>
+  </si>
+  <si>
+    <t>https://interop.esante.gouv.fr/ig/fhir/sdo/StructureDefinition/sdo-bundle-resultat-recherche-notification-esms</t>
+  </si>
+  <si>
+    <t>SDOBundleResultatRechercheNotificationESMS</t>
   </si>
   <si>
     <t>Profil pour la définition du Bundle de réponse à la recherche d'une notification</t>
   </si>
   <si>
-    <t xml:space="preserve">Resource {https://interop.esante.gouv.fr/ig/fhir/sdo/StructureDefinition/sdo-task}
-</t>
-  </si>
-  <si>
-    <t>dom-2:If the resource is contained in another resource, it SHALL NOT contain nested Resources {contained.contained.empty()}
-dom-4:If a resource is contained in another resource, it SHALL NOT have a meta.versionId or a meta.lastUpdated {contained.meta.versionId.empty() and contained.meta.lastUpdated.empty()}dom-3:If the resource is contained in another resource, it SHALL be referred to from elsewhere in the resource or SHALL refer to the containing resource {contained.where((('#'+id in (%resource.descendants().reference | %resource.descendants().as(canonical) | %resource.descendants().as(uri) | %resource.descendants().as(url))) or descendants().where(reference = '#').exists() or descendants().where(as(canonical) = '#').exists() or descendants().where(as(canonical) = '#').exists()).not()).trace('unmatched', id).empty()}dom-6:A resource should have narrative for robust management {text.`div`.exists()}dom-5:If a resource is contained in another resource, it SHALL NOT have a security label {contained.meta.security.empty()}inv-1:Last modified date must be greater than or equal to authored-on date. {lastModified.exists().not() or authoredOn.exists().not() or lastModified &gt;= authoredOn}</t>
+    <t>A resource in the bundle</t>
+  </si>
+  <si>
+    <t>The Resource for the entry. The purpose/meaning of the resource is determined by the Bundle.type.</t>
   </si>
 </sst>
 </file>
@@ -52865,16 +52863,16 @@
         <v>72</v>
       </c>
       <c r="K460" t="s" s="2">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="L460" t="s" s="2">
+        <v>255</v>
+      </c>
+      <c r="M460" t="s" s="2">
         <v>1110</v>
       </c>
-      <c r="M460" t="s" s="2">
-        <v>684</v>
-      </c>
       <c r="N460" t="s" s="2">
-        <v>685</v>
+        <v>1111</v>
       </c>
       <c r="O460" s="2"/>
       <c r="P460" s="2"/>
@@ -52937,7 +52935,7 @@
         <v>72</v>
       </c>
       <c r="AK460" t="s" s="2">
-        <v>1111</v>
+        <v>72</v>
       </c>
     </row>
     <row r="461">

</xml_diff>